<commit_message>
Add Simple Flow Round-3 Vendor Missing ordering bug draft (bug 5)
Adds the 2026-07-16 Milos-decision deviation to the bug-drafts deliverable:
Vendor Missing group renders at TOP of the WO Receive (Purchase Order
Details) screen but should sit at BOTTOM there; Bulk Receive (Receive
Vendor Parts) correctly keeps it at top. Live-observed 2026-07-16
(evidence in viu-round3-2026-07-16/). Affects SF-RCV-05 (C29373) and
SF-RCV-07 (C29375), both marked Deviation. Reader-facing text kept in
plain layman language (Standing Rule 7); SF-/C##### + evidence path in
the QA Internal Mapping sheet only. Regenerated via gen_bug_drafts_workbook.py.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Bug-Drafts.xlsx
+++ b/build/simple-flow/SimpleFlow_Bug-Drafts.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,7 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Four issues found while testing Simple Mode, written in plain English. Each row explains what happens now, what should happen instead, and simple steps to see it. (These are defects for the dev team - not questions for the product owner.)</t>
+          <t>Five issues found while testing Simple Mode, written in plain English. Each row explains what happens now, what should happen instead, and simple steps to see it. (These are defects for the dev team - not questions for the product owner.)</t>
         </is>
       </c>
     </row>
@@ -690,6 +690,40 @@
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="185" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>On the Receive screen, the "Vendor Missing" group of parts shows at the top instead of the bottom</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>When you open a work order and click the "Receive" button, you land on the "Purchase Order Details" screen, where the parts are grouped by supplier. Parts that don't have a supplier assigned yet are put in a "Vendor Missing" group. On this Receive screen that "Vendor Missing" group appears at the TOP of the list, above all the supplier groups. It has been agreed it should appear at the BOTTOM here. (On the separate "Bulk Receive" / "Receive Vendor Parts" page the "Vendor Missing" group correctly shows at the top - that page is fine and should not change.)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>On the Receive ("Purchase Order Details") screen reached from a work order's "Receive" button, the "Vendor Missing" group should appear at the BOTTOM of the list, below the supplier groups. The "Bulk Receive" / "Receive Vendor Parts" page should keep showing it at the top, unchanged.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>1. Open a work order that has some parts with a supplier and at least one part with no supplier assigned yet.
+2. Click the "Receive" button on the work order to open the "Purchase Order Details" screen.
+3. Look at where the "Vendor Missing" group sits in the list.
+4. Notice it is at the TOP, above the supplier groups - it should be at the BOTTOM here.
+5. For comparison, open the "Bulk Receive" / "Receive Vendor Parts" page and confirm the "Vendor Missing" group is at the top there - that one is correct.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -708,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1362,24 +1396,78 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Notes: Source of truth = jira-bug-drafts.md (4 active tickets TICKET 2-5, post-Milos-Round-2, updated 2026-07-10). TestRail IDs sourced from testrail-id-map.csv (standing rule 8). These are DEFECTS for the dev team (Jira TICKET 2-5 under epic SV-7301, Product Area Work Orders) - NOT filed yet (no Atlassian MCP here; file from the chat app). Kept OUT of any PO-facing deliverable (standing rule 7). DROPPED as expected: BUG-5/TICKET 1 (reviewer != completer descoped v1, Milos 2026-07-10). CLOSED / not filed: BUG-3 (review-note descoped, Milos R2 Q1), BUG-9/GAP-A (vendorless category-req/sell-optional intended, Milos R2 Q4), BUG-1/2/4/10.</t>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Round-3 deviation (Milos 2026-07-16 decision). No prior BUG-code; new dev ticket draft.</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>SF-RCV-05</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>C29373</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29373</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Refs: SV-7301 / Story 12 (Accept Delivery). Milos 2026-07-16: Vendor Missing group should sit at BOTTOM on the WO Receive (Purchase Order Details, grouped-by-vendor) surface but at TOP on the Bulk Receive (Receive Vendor Parts) page. Live-observed 2026-07-16: Vendor Missing renders at TOP on the WO Receive screen (wrong); TOP on Bulk Receive (correct). Evidence viu-round3-2026-07-16/ORDER-RECV-S15878-full.png, ORDER-RECV-S15878-Aeboro-miss.png (WO Receive) vs BULK-groups-full.png (Bulk Receive); observations.json.
+Status: OPEN — CONFIRMED deviation. Low (minor UI ordering per PO decision). SF-RCV-05 + SF-RCV-07 now marked Deviation. Bulk Receive surface is correct — no change there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>SF-RCV-07</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>C29375</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29375</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n"/>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Notes: Source of truth = jira-bug-drafts.md (4 active tickets TICKET 2-5, post-Milos-Round-2, updated 2026-07-10) PLUS bug 5, a Round-3 deviation (Milos 2026-07-16 decision; live-observed 2026-07-16). TestRail IDs sourced from testrail-id-map.csv (standing rule 8). These are DEFECTS for the dev team (Jira TICKET 2-5 + the Round-3 deviation under epic SV-7301, Product Area Work Orders) - NOT filed yet (no Atlassian MCP here; file from the chat app). Kept OUT of any PO-facing deliverable (standing rule 7). DROPPED as expected: BUG-5/TICKET 1 (reviewer != completer descoped v1, Milos 2026-07-10). CLOSED / not filed: BUG-3 (review-note descoped, Milos R2 Q1), BUG-9/GAP-A (vendorless category-req/sell-optional intended, Milos R2 Q4), BUG-1/2/4/10.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="14">
     <mergeCell ref="A8:A13"/>
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="F4:F7"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="F32:F33"/>
     <mergeCell ref="F8:F13"/>
+    <mergeCell ref="B32:B33"/>
     <mergeCell ref="F14:F30"/>
     <mergeCell ref="B4:B7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B8:B13"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A14:A30"/>
     <mergeCell ref="B14:B30"/>
   </mergeCells>
@@ -1412,6 +1500,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>